<commit_message>
feat: persist rent paid to previous owners across database, Excel templates, generator, and UI
</commit_message>
<xml_diff>
--- a/docs/4_Krishna_Valley_Previous_Owners_Dossier.xlsx
+++ b/docs/4_Krishna_Valley_Previous_Owners_Dossier.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S68"/>
+  <dimension ref="A1:V68"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -414,13 +414,16 @@
     <col min="10" max="10" width="21.83203125" customWidth="1"/>
     <col min="11" max="11" width="23.83203125" customWidth="1"/>
     <col min="12" max="12" width="25.83203125" customWidth="1"/>
-    <col min="13" max="13" width="27.83203125" customWidth="1"/>
-    <col min="14" max="14" width="35.83203125" customWidth="1"/>
-    <col min="15" max="15" width="22.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="19.83203125" customWidth="1"/>
-    <col min="18" max="18" width="14.83203125" customWidth="1"/>
-    <col min="19" max="19" width="45.83203125" customWidth="1"/>
+    <col min="13" max="13" width="40.83203125" customWidth="1"/>
+    <col min="14" max="14" width="34.83203125" customWidth="1"/>
+    <col min="15" max="15" width="29.83203125" customWidth="1"/>
+    <col min="16" max="16" width="31.83203125" customWidth="1"/>
+    <col min="17" max="17" width="35.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="19.83203125" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="45.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,24 +464,33 @@
         <v>Historical Paid Amount</v>
       </c>
       <c r="M1" t="str">
-        <v>Pre-Possession Rent Paid</v>
+        <v>Total Rent Paid to Previous Owner (₹)</v>
       </c>
       <c r="N1" t="str">
+        <v>Previous Owner Monthly Rent (₹)</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Previous Owner Paid Months</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Pre-Possession Rent Paid (₹)</v>
+      </c>
+      <c r="Q1" t="str">
         <v>Current Owner Name</v>
       </c>
-      <c r="O1" t="str">
+      <c r="R1" t="str">
         <v>Current Owner Phone</v>
       </c>
-      <c r="P1" t="str">
+      <c r="S1" t="str">
         <v>Bank Name</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="T1" t="str">
         <v>Account Number</v>
       </c>
-      <c r="R1" t="str">
+      <c r="U1" t="str">
         <v>IFSC Code</v>
       </c>
-      <c r="S1" t="str">
+      <c r="V1" t="str">
         <v>Remarks</v>
       </c>
     </row>
@@ -522,22 +534,31 @@
       <c r="M2">
         <v>0</v>
       </c>
-      <c r="N2" t="str">
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="str">
         <v>Padam Kumar &amp; Nitin Kumar</v>
       </c>
-      <c r="O2" t="str">
+      <c r="R2" t="str">
         <v>+91 9800000005</v>
       </c>
-      <c r="P2" t="str">
+      <c r="S2" t="str">
         <v/>
       </c>
-      <c r="Q2" t="str">
+      <c r="T2" t="str">
         <v/>
       </c>
-      <c r="R2" t="str">
+      <c r="U2" t="str">
         <v/>
       </c>
-      <c r="S2" t="str">
+      <c r="V2" t="str">
         <v>Resold title to Padam Kumar &amp; Nitin Kumar</v>
       </c>
     </row>
@@ -581,23 +602,32 @@
       <c r="M3">
         <v>1600000</v>
       </c>
-      <c r="N3" t="str">
+      <c r="N3">
+        <v>16000</v>
+      </c>
+      <c r="O3">
+        <v>100</v>
+      </c>
+      <c r="P3">
+        <v>1600000</v>
+      </c>
+      <c r="Q3" t="str">
         <v>Shakuntla Gupta</v>
       </c>
-      <c r="O3" t="str">
+      <c r="R3" t="str">
         <v>+91 9800000105</v>
       </c>
-      <c r="P3" t="str">
+      <c r="S3" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="T3" t="str">
         <v>0983000100182033</v>
       </c>
-      <c r="R3" t="str">
+      <c r="U3" t="str">
         <v>PUNB0098300</v>
       </c>
-      <c r="S3" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V3" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="4">
@@ -640,23 +670,32 @@
       <c r="M4">
         <v>1600000</v>
       </c>
-      <c r="N4" t="str">
+      <c r="N4">
+        <v>16000</v>
+      </c>
+      <c r="O4">
+        <v>100</v>
+      </c>
+      <c r="P4">
+        <v>1600000</v>
+      </c>
+      <c r="Q4" t="str">
         <v>MADAN GOPAL SARASWAT</v>
       </c>
-      <c r="O4" t="str">
+      <c r="R4" t="str">
         <v>+91 9800000105</v>
       </c>
-      <c r="P4" t="str">
+      <c r="S4" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="T4" t="str">
         <v>0983000100182033</v>
       </c>
-      <c r="R4" t="str">
+      <c r="U4" t="str">
         <v>PUNB0098300</v>
       </c>
-      <c r="S4" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V4" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="5">
@@ -699,22 +738,31 @@
       <c r="M5">
         <v>0</v>
       </c>
-      <c r="N5" t="str">
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="str">
         <v>Nitin Kumar</v>
       </c>
-      <c r="O5" t="str">
+      <c r="R5" t="str">
         <v>+91 9800000111</v>
       </c>
-      <c r="P5" t="str">
+      <c r="S5" t="str">
         <v/>
       </c>
-      <c r="Q5" t="str">
+      <c r="T5" t="str">
         <v/>
       </c>
-      <c r="R5" t="str">
+      <c r="U5" t="str">
         <v/>
       </c>
-      <c r="S5" t="str">
+      <c r="V5" t="str">
         <v>Resold title to Nitin Kumar</v>
       </c>
     </row>
@@ -758,23 +806,32 @@
       <c r="M6">
         <v>1568000</v>
       </c>
-      <c r="N6" t="str">
+      <c r="N6">
+        <v>16000</v>
+      </c>
+      <c r="O6">
+        <v>98</v>
+      </c>
+      <c r="P6">
+        <v>1568000</v>
+      </c>
+      <c r="Q6" t="str">
         <v>Shashi Bala</v>
       </c>
-      <c r="O6" t="str">
+      <c r="R6" t="str">
         <v>+91 9800000201</v>
       </c>
-      <c r="P6" t="str">
+      <c r="S6" t="str">
         <v>KMB</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="T6" t="str">
         <v>4711671610</v>
       </c>
-      <c r="R6" t="str">
+      <c r="U6" t="str">
         <v>KKBK0004632</v>
       </c>
-      <c r="S6" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1568000) - ajay</v>
+      <c r="V6" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1568000) - ajay</v>
       </c>
     </row>
     <row r="7">
@@ -817,23 +874,32 @@
       <c r="M7">
         <v>1600000</v>
       </c>
-      <c r="N7" t="str">
+      <c r="N7">
+        <v>16000</v>
+      </c>
+      <c r="O7">
+        <v>98</v>
+      </c>
+      <c r="P7">
+        <v>1600000</v>
+      </c>
+      <c r="Q7" t="str">
         <v>Sushil Kumar Burman</v>
       </c>
-      <c r="O7" t="str">
+      <c r="R7" t="str">
         <v>+91 9800000203</v>
       </c>
-      <c r="P7" t="str">
+      <c r="S7" t="str">
         <v>HDFC</v>
       </c>
-      <c r="Q7" t="str">
+      <c r="T7" t="str">
         <v>03281570006971</v>
       </c>
-      <c r="R7" t="str">
+      <c r="U7" t="str">
         <v>HDFC0000328</v>
       </c>
-      <c r="S7" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V7" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="8">
@@ -876,23 +942,32 @@
       <c r="M8">
         <v>1600000</v>
       </c>
-      <c r="N8" t="str">
+      <c r="N8">
+        <v>16000</v>
+      </c>
+      <c r="O8">
+        <v>98</v>
+      </c>
+      <c r="P8">
+        <v>1600000</v>
+      </c>
+      <c r="Q8" t="str">
         <v>Sarika Jain</v>
       </c>
-      <c r="O8" t="str">
+      <c r="R8" t="str">
         <v>+91 9800000203</v>
       </c>
-      <c r="P8" t="str">
+      <c r="S8" t="str">
         <v>HDFC</v>
       </c>
-      <c r="Q8" t="str">
+      <c r="T8" t="str">
         <v>03281570006971</v>
       </c>
-      <c r="R8" t="str">
+      <c r="U8" t="str">
         <v>HDFC0000328</v>
       </c>
-      <c r="S8" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V8" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="9">
@@ -935,23 +1010,32 @@
       <c r="M9">
         <v>1600000</v>
       </c>
-      <c r="N9" t="str">
+      <c r="N9">
+        <v>16000</v>
+      </c>
+      <c r="O9">
+        <v>100</v>
+      </c>
+      <c r="P9">
+        <v>1600000</v>
+      </c>
+      <c r="Q9" t="str">
         <v>Asha Mishra</v>
       </c>
-      <c r="O9" t="str">
+      <c r="R9" t="str">
         <v>+91 9800000205</v>
       </c>
-      <c r="P9" t="str">
+      <c r="S9" t="str">
         <v>BOB</v>
       </c>
-      <c r="Q9" t="str">
+      <c r="T9" t="str">
         <v>40790100002749</v>
       </c>
-      <c r="R9" t="str">
+      <c r="U9" t="str">
         <v>BARB0SHAMSH</v>
       </c>
-      <c r="S9" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V9" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="10">
@@ -994,23 +1078,32 @@
       <c r="M10">
         <v>1600000</v>
       </c>
-      <c r="N10" t="str">
+      <c r="N10">
+        <v>16000</v>
+      </c>
+      <c r="O10">
+        <v>100</v>
+      </c>
+      <c r="P10">
+        <v>1600000</v>
+      </c>
+      <c r="Q10" t="str">
         <v>Nirmala Devi</v>
       </c>
-      <c r="O10" t="str">
+      <c r="R10" t="str">
         <v>+91 9800000205</v>
       </c>
-      <c r="P10" t="str">
+      <c r="S10" t="str">
         <v>BOB</v>
       </c>
-      <c r="Q10" t="str">
+      <c r="T10" t="str">
         <v>40790100002749</v>
       </c>
-      <c r="R10" t="str">
+      <c r="U10" t="str">
         <v>BARB0SHAMSH</v>
       </c>
-      <c r="S10" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V10" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="11">
@@ -1053,23 +1146,32 @@
       <c r="M11">
         <v>1568000</v>
       </c>
-      <c r="N11" t="str">
+      <c r="N11">
+        <v>16000</v>
+      </c>
+      <c r="O11">
+        <v>98</v>
+      </c>
+      <c r="P11">
+        <v>1568000</v>
+      </c>
+      <c r="Q11" t="str">
         <v>Sukrit Gupta</v>
       </c>
-      <c r="O11" t="str">
+      <c r="R11" t="str">
         <v>+91 9800000213</v>
       </c>
-      <c r="P11" t="str">
+      <c r="S11" t="str">
         <v>IDBI</v>
       </c>
-      <c r="Q11" t="str">
+      <c r="T11" t="str">
         <v>193104000007276</v>
       </c>
-      <c r="R11" t="str">
+      <c r="U11" t="str">
         <v>IBKL0000193</v>
       </c>
-      <c r="S11" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1568000) - home</v>
+      <c r="V11" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1568000) - home</v>
       </c>
     </row>
     <row r="12">
@@ -1112,23 +1214,32 @@
       <c r="M12">
         <v>896000</v>
       </c>
-      <c r="N12" t="str">
+      <c r="N12">
+        <v>16000</v>
+      </c>
+      <c r="O12">
+        <v>56</v>
+      </c>
+      <c r="P12">
+        <v>896000</v>
+      </c>
+      <c r="Q12" t="str">
         <v>Madhu Bhandari</v>
       </c>
-      <c r="O12" t="str">
+      <c r="R12" t="str">
         <v>+91 9800000302</v>
       </c>
-      <c r="P12" t="str">
+      <c r="S12" t="str">
         <v>FBL</v>
       </c>
-      <c r="Q12" t="str">
+      <c r="T12" t="str">
         <v>16770100014919</v>
       </c>
-      <c r="R12" t="str">
+      <c r="U12" t="str">
         <v>FDRL0001677</v>
       </c>
-      <c r="S12" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹896000) - Clear</v>
+      <c r="V12" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹896000) - Clear</v>
       </c>
     </row>
     <row r="13">
@@ -1171,23 +1282,32 @@
       <c r="M13">
         <v>1600000</v>
       </c>
-      <c r="N13" t="str">
+      <c r="N13">
+        <v>16000</v>
+      </c>
+      <c r="O13">
+        <v>100</v>
+      </c>
+      <c r="P13">
+        <v>1600000</v>
+      </c>
+      <c r="Q13" t="str">
         <v>Rajender Pratap Singh</v>
       </c>
-      <c r="O13" t="str">
+      <c r="R13" t="str">
         <v>+91 9800000309</v>
       </c>
-      <c r="P13" t="str">
+      <c r="S13" t="str">
         <v>UBI</v>
       </c>
-      <c r="Q13" t="str">
+      <c r="T13" t="str">
         <v>302802011001470</v>
       </c>
-      <c r="R13" t="str">
+      <c r="U13" t="str">
         <v>UBIN0530263</v>
       </c>
-      <c r="S13" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - clear</v>
+      <c r="V13" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - clear</v>
       </c>
     </row>
     <row r="14">
@@ -1230,23 +1350,32 @@
       <c r="M14">
         <v>848000</v>
       </c>
-      <c r="N14" t="str">
+      <c r="N14">
+        <v>16000</v>
+      </c>
+      <c r="O14">
+        <v>53</v>
+      </c>
+      <c r="P14">
+        <v>848000</v>
+      </c>
+      <c r="Q14" t="str">
         <v>Neeru Arora</v>
       </c>
-      <c r="O14" t="str">
+      <c r="R14" t="str">
         <v>+91 9800000314</v>
       </c>
-      <c r="P14" t="str">
+      <c r="S14" t="str">
         <v>KMB</v>
       </c>
-      <c r="Q14" t="str">
+      <c r="T14" t="str">
         <v>0211207458</v>
       </c>
-      <c r="R14" t="str">
+      <c r="U14" t="str">
         <v>KKBK0000216</v>
       </c>
-      <c r="S14" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹848000) - Clear</v>
+      <c r="V14" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹848000) - Clear</v>
       </c>
     </row>
     <row r="15">
@@ -1289,23 +1418,32 @@
       <c r="M15">
         <v>848000</v>
       </c>
-      <c r="N15" t="str">
+      <c r="N15">
+        <v>16000</v>
+      </c>
+      <c r="O15">
+        <v>53</v>
+      </c>
+      <c r="P15">
+        <v>848000</v>
+      </c>
+      <c r="Q15" t="str">
         <v>Gaurav Gupta</v>
       </c>
-      <c r="O15" t="str">
+      <c r="R15" t="str">
         <v>+91 9800000314</v>
       </c>
-      <c r="P15" t="str">
+      <c r="S15" t="str">
         <v>KMB</v>
       </c>
-      <c r="Q15" t="str">
+      <c r="T15" t="str">
         <v>0211207458</v>
       </c>
-      <c r="R15" t="str">
+      <c r="U15" t="str">
         <v>KKBK0000216</v>
       </c>
-      <c r="S15" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹848000) - Clear</v>
+      <c r="V15" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹848000) - Clear</v>
       </c>
     </row>
     <row r="16">
@@ -1348,23 +1486,32 @@
       <c r="M16">
         <v>1600000</v>
       </c>
-      <c r="N16" t="str">
+      <c r="N16">
+        <v>16000</v>
+      </c>
+      <c r="O16">
+        <v>100</v>
+      </c>
+      <c r="P16">
+        <v>1600000</v>
+      </c>
+      <c r="Q16" t="str">
         <v>Anita Gupta</v>
       </c>
-      <c r="O16" t="str">
+      <c r="R16" t="str">
         <v>+91 9800000403</v>
       </c>
-      <c r="P16" t="str">
+      <c r="S16" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q16" t="str">
+      <c r="T16" t="str">
         <v>628701020108</v>
       </c>
-      <c r="R16" t="str">
+      <c r="U16" t="str">
         <v>ICIC0006287</v>
       </c>
-      <c r="S16" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V16" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="17">
@@ -1407,23 +1554,32 @@
       <c r="M17">
         <v>1600000</v>
       </c>
-      <c r="N17" t="str">
+      <c r="N17">
+        <v>16000</v>
+      </c>
+      <c r="O17">
+        <v>100</v>
+      </c>
+      <c r="P17">
+        <v>1600000</v>
+      </c>
+      <c r="Q17" t="str">
         <v>Anita Gupta</v>
       </c>
-      <c r="O17" t="str">
+      <c r="R17" t="str">
         <v>+91 9800000403</v>
       </c>
-      <c r="P17" t="str">
+      <c r="S17" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q17" t="str">
+      <c r="T17" t="str">
         <v>628701020108</v>
       </c>
-      <c r="R17" t="str">
+      <c r="U17" t="str">
         <v>ICIC0006287</v>
       </c>
-      <c r="S17" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V17" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="18">
@@ -1466,23 +1622,32 @@
       <c r="M18">
         <v>1600000</v>
       </c>
-      <c r="N18" t="str">
+      <c r="N18">
+        <v>16000</v>
+      </c>
+      <c r="O18">
+        <v>100</v>
+      </c>
+      <c r="P18">
+        <v>1600000</v>
+      </c>
+      <c r="Q18" t="str">
         <v>Anita Gupta</v>
       </c>
-      <c r="O18" t="str">
+      <c r="R18" t="str">
         <v>+91 9800000403</v>
       </c>
-      <c r="P18" t="str">
+      <c r="S18" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q18" t="str">
+      <c r="T18" t="str">
         <v>628701020108</v>
       </c>
-      <c r="R18" t="str">
+      <c r="U18" t="str">
         <v>ICIC0006287</v>
       </c>
-      <c r="S18" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V18" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="19">
@@ -1525,23 +1690,32 @@
       <c r="M19">
         <v>656000</v>
       </c>
-      <c r="N19" t="str">
+      <c r="N19">
+        <v>16000</v>
+      </c>
+      <c r="O19">
+        <v>41</v>
+      </c>
+      <c r="P19">
+        <v>656000</v>
+      </c>
+      <c r="Q19" t="str">
         <v>Suman Rani</v>
       </c>
-      <c r="O19" t="str">
+      <c r="R19" t="str">
         <v>+91 9800000404</v>
       </c>
-      <c r="P19" t="str">
+      <c r="S19" t="str">
         <v>ARYAVART</v>
       </c>
-      <c r="Q19" t="str">
+      <c r="T19" t="str">
         <v>120510100003455</v>
       </c>
-      <c r="R19" t="str">
+      <c r="U19" t="str">
         <v>BKID0ARYAGB</v>
       </c>
-      <c r="S19" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹656000) - canara bank neeraj ji</v>
+      <c r="V19" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹656000) - canara bank neeraj ji</v>
       </c>
     </row>
     <row r="20">
@@ -1584,23 +1758,32 @@
       <c r="M20">
         <v>656000</v>
       </c>
-      <c r="N20" t="str">
+      <c r="N20">
+        <v>16000</v>
+      </c>
+      <c r="O20">
+        <v>41</v>
+      </c>
+      <c r="P20">
+        <v>656000</v>
+      </c>
+      <c r="Q20" t="str">
         <v>Vishnu Kumar Agarwal</v>
       </c>
-      <c r="O20" t="str">
+      <c r="R20" t="str">
         <v>+91 9800000404</v>
       </c>
-      <c r="P20" t="str">
+      <c r="S20" t="str">
         <v>ARYAVART</v>
       </c>
-      <c r="Q20" t="str">
+      <c r="T20" t="str">
         <v>120510100003455</v>
       </c>
-      <c r="R20" t="str">
+      <c r="U20" t="str">
         <v>BKID0ARYAGB</v>
       </c>
-      <c r="S20" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹656000) - canara bank neeraj ji</v>
+      <c r="V20" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹656000) - canara bank neeraj ji</v>
       </c>
     </row>
     <row r="21">
@@ -1643,23 +1826,32 @@
       <c r="M21">
         <v>512000</v>
       </c>
-      <c r="N21" t="str">
+      <c r="N21">
+        <v>16000</v>
+      </c>
+      <c r="O21">
+        <v>32</v>
+      </c>
+      <c r="P21">
+        <v>512000</v>
+      </c>
+      <c r="Q21" t="str">
         <v>Ketiki Singh Shastri</v>
       </c>
-      <c r="O21" t="str">
+      <c r="R21" t="str">
         <v>+91 9800000408</v>
       </c>
-      <c r="P21" t="str">
+      <c r="S21" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q21" t="str">
+      <c r="T21" t="str">
         <v>696501700139</v>
       </c>
-      <c r="R21" t="str">
+      <c r="U21" t="str">
         <v>ICIC0006965</v>
       </c>
-      <c r="S21" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹512000) - bank</v>
+      <c r="V21" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹512000) - bank</v>
       </c>
     </row>
     <row r="22">
@@ -1702,23 +1894,32 @@
       <c r="M22">
         <v>688000</v>
       </c>
-      <c r="N22" t="str">
+      <c r="N22">
+        <v>16000</v>
+      </c>
+      <c r="O22">
+        <v>43</v>
+      </c>
+      <c r="P22">
+        <v>688000</v>
+      </c>
+      <c r="Q22" t="str">
         <v>Manju Arora</v>
       </c>
-      <c r="O22" t="str">
+      <c r="R22" t="str">
         <v>+91 9800000410</v>
       </c>
-      <c r="P22" t="str">
+      <c r="S22" t="str">
         <v>AXIS</v>
       </c>
-      <c r="Q22" t="str">
+      <c r="T22" t="str">
         <v>918010087348090</v>
       </c>
-      <c r="R22" t="str">
+      <c r="U22" t="str">
         <v>UTIB0003958</v>
       </c>
-      <c r="S22" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹688000) - Clear</v>
+      <c r="V22" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹688000) - Clear</v>
       </c>
     </row>
     <row r="23">
@@ -1761,23 +1962,32 @@
       <c r="M23">
         <v>688000</v>
       </c>
-      <c r="N23" t="str">
+      <c r="N23">
+        <v>16000</v>
+      </c>
+      <c r="O23">
+        <v>43</v>
+      </c>
+      <c r="P23">
+        <v>688000</v>
+      </c>
+      <c r="Q23" t="str">
         <v>Mamta Singh</v>
       </c>
-      <c r="O23" t="str">
+      <c r="R23" t="str">
         <v>+91 9800000410</v>
       </c>
-      <c r="P23" t="str">
+      <c r="S23" t="str">
         <v>AXIS</v>
       </c>
-      <c r="Q23" t="str">
+      <c r="T23" t="str">
         <v>918010087348090</v>
       </c>
-      <c r="R23" t="str">
+      <c r="U23" t="str">
         <v>UTIB0003958</v>
       </c>
-      <c r="S23" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹688000) - Clear</v>
+      <c r="V23" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹688000) - Clear</v>
       </c>
     </row>
     <row r="24">
@@ -1820,23 +2030,32 @@
       <c r="M24">
         <v>624000</v>
       </c>
-      <c r="N24" t="str">
+      <c r="N24">
+        <v>16000</v>
+      </c>
+      <c r="O24">
+        <v>39</v>
+      </c>
+      <c r="P24">
+        <v>624000</v>
+      </c>
+      <c r="Q24" t="str">
         <v>Sushma Jain</v>
       </c>
-      <c r="O24" t="str">
+      <c r="R24" t="str">
         <v>+91 9800000411</v>
       </c>
-      <c r="P24" t="str">
+      <c r="S24" t="str">
         <v>AXIS</v>
       </c>
-      <c r="Q24" t="str">
+      <c r="T24" t="str">
         <v>086010100282369</v>
       </c>
-      <c r="R24" t="str">
+      <c r="U24" t="str">
         <v>UTIB0000086</v>
       </c>
-      <c r="S24" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹624000) - Clear</v>
+      <c r="V24" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹624000) - Clear</v>
       </c>
     </row>
     <row r="25">
@@ -1879,23 +2098,32 @@
       <c r="M25">
         <v>624000</v>
       </c>
-      <c r="N25" t="str">
+      <c r="N25">
+        <v>16000</v>
+      </c>
+      <c r="O25">
+        <v>39</v>
+      </c>
+      <c r="P25">
+        <v>624000</v>
+      </c>
+      <c r="Q25" t="str">
         <v>SWATI</v>
       </c>
-      <c r="O25" t="str">
+      <c r="R25" t="str">
         <v>+91 9800000411</v>
       </c>
-      <c r="P25" t="str">
+      <c r="S25" t="str">
         <v>AXIS</v>
       </c>
-      <c r="Q25" t="str">
+      <c r="T25" t="str">
         <v>086010100282369</v>
       </c>
-      <c r="R25" t="str">
+      <c r="U25" t="str">
         <v>UTIB0000086</v>
       </c>
-      <c r="S25" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹624000) - Clear</v>
+      <c r="V25" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹624000) - Clear</v>
       </c>
     </row>
     <row r="26">
@@ -1938,23 +2166,32 @@
       <c r="M26">
         <v>672000</v>
       </c>
-      <c r="N26" t="str">
+      <c r="N26">
+        <v>16000</v>
+      </c>
+      <c r="O26">
+        <v>42</v>
+      </c>
+      <c r="P26">
+        <v>672000</v>
+      </c>
+      <c r="Q26" t="str">
         <v>Geeta Giri</v>
       </c>
-      <c r="O26" t="str">
+      <c r="R26" t="str">
         <v>+91 9800000413</v>
       </c>
-      <c r="P26" t="str">
+      <c r="S26" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q26" t="str">
+      <c r="T26" t="str">
         <v>4955000100030984</v>
       </c>
-      <c r="R26" t="str">
+      <c r="U26" t="str">
         <v>PUNB0495500</v>
       </c>
-      <c r="S26" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹672000) - Clear</v>
+      <c r="V26" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹672000) - Clear</v>
       </c>
     </row>
     <row r="27">
@@ -1997,23 +2234,32 @@
       <c r="M27">
         <v>672000</v>
       </c>
-      <c r="N27" t="str">
+      <c r="N27">
+        <v>16000</v>
+      </c>
+      <c r="O27">
+        <v>42</v>
+      </c>
+      <c r="P27">
+        <v>672000</v>
+      </c>
+      <c r="Q27" t="str">
         <v>Geeta Giri</v>
       </c>
-      <c r="O27" t="str">
+      <c r="R27" t="str">
         <v>+91 9800000413</v>
       </c>
-      <c r="P27" t="str">
+      <c r="S27" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q27" t="str">
+      <c r="T27" t="str">
         <v>4955000100030984</v>
       </c>
-      <c r="R27" t="str">
+      <c r="U27" t="str">
         <v>PUNB0495500</v>
       </c>
-      <c r="S27" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹672000) - Clear</v>
+      <c r="V27" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹672000) - Clear</v>
       </c>
     </row>
     <row r="28">
@@ -2056,23 +2302,32 @@
       <c r="M28">
         <v>672000</v>
       </c>
-      <c r="N28" t="str">
+      <c r="N28">
+        <v>16000</v>
+      </c>
+      <c r="O28">
+        <v>42</v>
+      </c>
+      <c r="P28">
+        <v>672000</v>
+      </c>
+      <c r="Q28" t="str">
         <v>GEETA GIRI</v>
       </c>
-      <c r="O28" t="str">
+      <c r="R28" t="str">
         <v>+91 9800000413</v>
       </c>
-      <c r="P28" t="str">
+      <c r="S28" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q28" t="str">
+      <c r="T28" t="str">
         <v>4955000100030984</v>
       </c>
-      <c r="R28" t="str">
+      <c r="U28" t="str">
         <v>PUNB0495500</v>
       </c>
-      <c r="S28" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹672000) - Clear</v>
+      <c r="V28" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹672000) - Clear</v>
       </c>
     </row>
     <row r="29">
@@ -2115,23 +2370,32 @@
       <c r="M29">
         <v>1600000</v>
       </c>
-      <c r="N29" t="str">
+      <c r="N29">
+        <v>16000</v>
+      </c>
+      <c r="O29">
+        <v>100</v>
+      </c>
+      <c r="P29">
+        <v>1600000</v>
+      </c>
+      <c r="Q29" t="str">
         <v>Santokh Singh</v>
       </c>
-      <c r="O29" t="str">
+      <c r="R29" t="str">
         <v>+91 9800000501</v>
       </c>
-      <c r="P29" t="str">
+      <c r="S29" t="str">
         <v>KBL</v>
       </c>
-      <c r="Q29" t="str">
+      <c r="T29" t="str">
         <v>0302500100238001</v>
       </c>
-      <c r="R29" t="str">
+      <c r="U29" t="str">
         <v>KARB0000030</v>
       </c>
-      <c r="S29" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V29" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="30">
@@ -2174,23 +2438,32 @@
       <c r="M30">
         <v>1600000</v>
       </c>
-      <c r="N30" t="str">
+      <c r="N30">
+        <v>16000</v>
+      </c>
+      <c r="O30">
+        <v>100</v>
+      </c>
+      <c r="P30">
+        <v>1600000</v>
+      </c>
+      <c r="Q30" t="str">
         <v>Sunita Gupta</v>
       </c>
-      <c r="O30" t="str">
+      <c r="R30" t="str">
         <v>+91 9800000501</v>
       </c>
-      <c r="P30" t="str">
+      <c r="S30" t="str">
         <v>KBL</v>
       </c>
-      <c r="Q30" t="str">
+      <c r="T30" t="str">
         <v>0302500100238001</v>
       </c>
-      <c r="R30" t="str">
+      <c r="U30" t="str">
         <v>KARB0000030</v>
       </c>
-      <c r="S30" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V30" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="31">
@@ -2233,23 +2506,32 @@
       <c r="M31">
         <v>1600000</v>
       </c>
-      <c r="N31" t="str">
+      <c r="N31">
+        <v>16000</v>
+      </c>
+      <c r="O31">
+        <v>100</v>
+      </c>
+      <c r="P31">
+        <v>1600000</v>
+      </c>
+      <c r="Q31" t="str">
         <v>Shefali Rani Mukherji</v>
       </c>
-      <c r="O31" t="str">
+      <c r="R31" t="str">
         <v>+91 9800000503</v>
       </c>
-      <c r="P31" t="str">
+      <c r="S31" t="str">
         <v>SBI</v>
       </c>
-      <c r="Q31" t="str">
+      <c r="T31" t="str">
         <v>10932825848</v>
       </c>
-      <c r="R31" t="str">
+      <c r="U31" t="str">
         <v>SBIN0001076</v>
       </c>
-      <c r="S31" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V31" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="32">
@@ -2292,23 +2574,32 @@
       <c r="M32">
         <v>1600000</v>
       </c>
-      <c r="N32" t="str">
+      <c r="N32">
+        <v>16000</v>
+      </c>
+      <c r="O32">
+        <v>100</v>
+      </c>
+      <c r="P32">
+        <v>1600000</v>
+      </c>
+      <c r="Q32" t="str">
         <v>Manju Goyal</v>
       </c>
-      <c r="O32" t="str">
+      <c r="R32" t="str">
         <v>+91 9800000503</v>
       </c>
-      <c r="P32" t="str">
+      <c r="S32" t="str">
         <v>SBI</v>
       </c>
-      <c r="Q32" t="str">
+      <c r="T32" t="str">
         <v>10932825848</v>
       </c>
-      <c r="R32" t="str">
+      <c r="U32" t="str">
         <v>SBIN0001076</v>
       </c>
-      <c r="S32" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V32" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="33">
@@ -2351,23 +2642,32 @@
       <c r="M33">
         <v>608000</v>
       </c>
-      <c r="N33" t="str">
+      <c r="N33">
+        <v>16000</v>
+      </c>
+      <c r="O33">
+        <v>38</v>
+      </c>
+      <c r="P33">
+        <v>608000</v>
+      </c>
+      <c r="Q33" t="str">
         <v>Veena Sahani</v>
       </c>
-      <c r="O33" t="str">
+      <c r="R33" t="str">
         <v>+91 9800000507</v>
       </c>
-      <c r="P33" t="str">
+      <c r="S33" t="str">
         <v>BOB</v>
       </c>
-      <c r="Q33" t="str">
+      <c r="T33" t="str">
         <v>32200100000680</v>
       </c>
-      <c r="R33" t="str">
+      <c r="U33" t="str">
         <v>BARB0TILDEL</v>
       </c>
-      <c r="S33" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹608000) - Completed</v>
+      <c r="V33" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹608000) - Completed</v>
       </c>
     </row>
     <row r="34">
@@ -2410,23 +2710,32 @@
       <c r="M34">
         <v>608000</v>
       </c>
-      <c r="N34" t="str">
+      <c r="N34">
+        <v>16000</v>
+      </c>
+      <c r="O34">
+        <v>38</v>
+      </c>
+      <c r="P34">
+        <v>608000</v>
+      </c>
+      <c r="Q34" t="str">
         <v>Veena Sahani</v>
       </c>
-      <c r="O34" t="str">
+      <c r="R34" t="str">
         <v>+91 9800000507</v>
       </c>
-      <c r="P34" t="str">
+      <c r="S34" t="str">
         <v>BOB</v>
       </c>
-      <c r="Q34" t="str">
+      <c r="T34" t="str">
         <v>32200100000680</v>
       </c>
-      <c r="R34" t="str">
+      <c r="U34" t="str">
         <v>BARB0TILDEL</v>
       </c>
-      <c r="S34" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹608000) - Completed</v>
+      <c r="V34" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹608000) - Completed</v>
       </c>
     </row>
     <row r="35">
@@ -2469,23 +2778,32 @@
       <c r="M35">
         <v>1600000</v>
       </c>
-      <c r="N35" t="str">
+      <c r="N35">
+        <v>16000</v>
+      </c>
+      <c r="O35">
+        <v>100</v>
+      </c>
+      <c r="P35">
+        <v>1600000</v>
+      </c>
+      <c r="Q35" t="str">
         <v>Sanjay Madan and Sandhya Madan</v>
       </c>
-      <c r="O35" t="str">
+      <c r="R35" t="str">
         <v>+91 9800000508</v>
       </c>
-      <c r="P35" t="str">
+      <c r="S35" t="str">
         <v>CNB</v>
       </c>
-      <c r="Q35" t="str">
+      <c r="T35" t="str">
         <v>0378101083927</v>
       </c>
-      <c r="R35" t="str">
+      <c r="U35" t="str">
         <v>CNRB0002946</v>
       </c>
-      <c r="S35" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V35" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="36">
@@ -2528,23 +2846,32 @@
       <c r="M36">
         <v>1600000</v>
       </c>
-      <c r="N36" t="str">
+      <c r="N36">
+        <v>16000</v>
+      </c>
+      <c r="O36">
+        <v>100</v>
+      </c>
+      <c r="P36">
+        <v>1600000</v>
+      </c>
+      <c r="Q36" t="str">
         <v>Vishnu Kumar Agarwal</v>
       </c>
-      <c r="O36" t="str">
+      <c r="R36" t="str">
         <v>+91 9800000508</v>
       </c>
-      <c r="P36" t="str">
+      <c r="S36" t="str">
         <v>CNB</v>
       </c>
-      <c r="Q36" t="str">
+      <c r="T36" t="str">
         <v>0378101083927</v>
       </c>
-      <c r="R36" t="str">
+      <c r="U36" t="str">
         <v>CNRB0002946</v>
       </c>
-      <c r="S36" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V36" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="37">
@@ -2587,23 +2914,32 @@
       <c r="M37">
         <v>512000</v>
       </c>
-      <c r="N37" t="str">
+      <c r="N37">
+        <v>16000</v>
+      </c>
+      <c r="O37">
+        <v>32</v>
+      </c>
+      <c r="P37">
+        <v>512000</v>
+      </c>
+      <c r="Q37" t="str">
         <v>Prem Chand Gupta</v>
       </c>
-      <c r="O37" t="str">
+      <c r="R37" t="str">
         <v>+91 9800000513</v>
       </c>
-      <c r="P37" t="str">
+      <c r="S37" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q37" t="str">
+      <c r="T37" t="str">
         <v>4046000100000601</v>
       </c>
-      <c r="R37" t="str">
+      <c r="U37" t="str">
         <v>PUNB0404600</v>
       </c>
-      <c r="S37" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹512000) - bank</v>
+      <c r="V37" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹512000) - bank</v>
       </c>
     </row>
     <row r="38">
@@ -2646,23 +2982,32 @@
       <c r="M38">
         <v>512000</v>
       </c>
-      <c r="N38" t="str">
+      <c r="N38">
+        <v>16000</v>
+      </c>
+      <c r="O38">
+        <v>32</v>
+      </c>
+      <c r="P38">
+        <v>512000</v>
+      </c>
+      <c r="Q38" t="str">
         <v>Rani Gupta</v>
       </c>
-      <c r="O38" t="str">
+      <c r="R38" t="str">
         <v>+91 9800000514</v>
       </c>
-      <c r="P38" t="str">
+      <c r="S38" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q38" t="str">
+      <c r="T38" t="str">
         <v>2961000100008083</v>
       </c>
-      <c r="R38" t="str">
+      <c r="U38" t="str">
         <v>PUNB0296100</v>
       </c>
-      <c r="S38" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹512000) - bank</v>
+      <c r="V38" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹512000) - bank</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -2706,24 +3051,33 @@
       <c r="M39">
         <v>592000</v>
       </c>
-      <c r="N39" t="str" xml:space="preserve">
+      <c r="N39">
+        <v>16000</v>
+      </c>
+      <c r="O39">
+        <v>37</v>
+      </c>
+      <c r="P39">
+        <v>592000</v>
+      </c>
+      <c r="Q39" t="str" xml:space="preserve">
         <v xml:space="preserve">Rajesh Sharma _x000d_
 Kamlesh Sharma</v>
       </c>
-      <c r="O39" t="str">
+      <c r="R39" t="str">
         <v>+91 9800000601</v>
       </c>
-      <c r="P39" t="str">
+      <c r="S39" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q39" t="str">
+      <c r="T39" t="str">
         <v>153901503569</v>
       </c>
-      <c r="R39" t="str">
+      <c r="U39" t="str">
         <v>ICIC0001539</v>
       </c>
-      <c r="S39" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹592000) - hdfc / icici</v>
+      <c r="V39" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹592000) - hdfc / icici</v>
       </c>
     </row>
     <row r="40">
@@ -2766,23 +3120,32 @@
       <c r="M40">
         <v>656000</v>
       </c>
-      <c r="N40" t="str">
+      <c r="N40">
+        <v>16000</v>
+      </c>
+      <c r="O40">
+        <v>41</v>
+      </c>
+      <c r="P40">
+        <v>656000</v>
+      </c>
+      <c r="Q40" t="str">
         <v>Madhav Katara</v>
       </c>
-      <c r="O40" t="str">
+      <c r="R40" t="str">
         <v>+91 9800000602</v>
       </c>
-      <c r="P40" t="str">
+      <c r="S40" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q40" t="str">
+      <c r="T40" t="str">
         <v>156701500082</v>
       </c>
-      <c r="R40" t="str">
+      <c r="U40" t="str">
         <v>ICIC0001567</v>
       </c>
-      <c r="S40" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹656000) - Completed</v>
+      <c r="V40" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹656000) - Completed</v>
       </c>
     </row>
     <row r="41">
@@ -2825,23 +3188,32 @@
       <c r="M41">
         <v>1488000</v>
       </c>
-      <c r="N41" t="str">
+      <c r="N41">
+        <v>16000</v>
+      </c>
+      <c r="O41">
+        <v>93</v>
+      </c>
+      <c r="P41">
+        <v>1488000</v>
+      </c>
+      <c r="Q41" t="str">
         <v>Akshay Khullar</v>
       </c>
-      <c r="O41" t="str">
+      <c r="R41" t="str">
         <v>+91 9800000603</v>
       </c>
-      <c r="P41" t="str">
+      <c r="S41" t="str">
         <v>KMB</v>
       </c>
-      <c r="Q41" t="str">
+      <c r="T41" t="str">
         <v>5811122361</v>
       </c>
-      <c r="R41" t="str">
+      <c r="U41" t="str">
         <v>KKBK0000182</v>
       </c>
-      <c r="S41" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1488000) - Completed</v>
+      <c r="V41" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1488000) - Completed</v>
       </c>
     </row>
     <row r="42">
@@ -2884,23 +3256,32 @@
       <c r="M42">
         <v>1488000</v>
       </c>
-      <c r="N42" t="str">
+      <c r="N42">
+        <v>16000</v>
+      </c>
+      <c r="O42">
+        <v>93</v>
+      </c>
+      <c r="P42">
+        <v>1488000</v>
+      </c>
+      <c r="Q42" t="str">
         <v>Pooja Chand Dwivedi</v>
       </c>
-      <c r="O42" t="str">
+      <c r="R42" t="str">
         <v>+91 9800000603</v>
       </c>
-      <c r="P42" t="str">
+      <c r="S42" t="str">
         <v>KMB</v>
       </c>
-      <c r="Q42" t="str">
+      <c r="T42" t="str">
         <v>5811122361</v>
       </c>
-      <c r="R42" t="str">
+      <c r="U42" t="str">
         <v>KKBK0000182</v>
       </c>
-      <c r="S42" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1488000) - Completed</v>
+      <c r="V42" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1488000) - Completed</v>
       </c>
     </row>
     <row r="43">
@@ -2943,22 +3324,31 @@
       <c r="M43">
         <v>112000</v>
       </c>
-      <c r="N43" t="str">
+      <c r="N43">
+        <v>16000</v>
+      </c>
+      <c r="O43">
+        <v>7</v>
+      </c>
+      <c r="P43">
+        <v>112000</v>
+      </c>
+      <c r="Q43" t="str">
         <v>Prateek Bansal</v>
       </c>
-      <c r="O43" t="str">
+      <c r="R43" t="str">
         <v>+91 9800000609</v>
       </c>
-      <c r="P43" t="str">
+      <c r="S43" t="str">
         <v>HDFC</v>
       </c>
-      <c r="Q43" t="str">
+      <c r="T43" t="str">
         <v>01211000273675</v>
       </c>
-      <c r="R43" t="str">
+      <c r="U43" t="str">
         <v>HDFC0000121</v>
       </c>
-      <c r="S43" t="str">
+      <c r="V43" t="str">
         <v>Historical title archive</v>
       </c>
     </row>
@@ -3002,23 +3392,32 @@
       <c r="M44">
         <v>704000</v>
       </c>
-      <c r="N44" t="str">
+      <c r="N44">
+        <v>16000</v>
+      </c>
+      <c r="O44">
+        <v>44</v>
+      </c>
+      <c r="P44">
+        <v>704000</v>
+      </c>
+      <c r="Q44" t="str">
         <v>Jitender Kumar</v>
       </c>
-      <c r="O44" t="str">
+      <c r="R44" t="str">
         <v>+91 9800000610</v>
       </c>
-      <c r="P44" t="str">
+      <c r="S44" t="str">
         <v>CBI</v>
       </c>
-      <c r="Q44" t="str">
+      <c r="T44" t="str">
         <v>1075835628</v>
       </c>
-      <c r="R44" t="str">
+      <c r="U44" t="str">
         <v>CBIN0281467</v>
       </c>
-      <c r="S44" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹704000) - Clear</v>
+      <c r="V44" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹704000) - Clear</v>
       </c>
     </row>
     <row r="45">
@@ -3061,23 +3460,32 @@
       <c r="M45">
         <v>704000</v>
       </c>
-      <c r="N45" t="str">
+      <c r="N45">
+        <v>16000</v>
+      </c>
+      <c r="O45">
+        <v>44</v>
+      </c>
+      <c r="P45">
+        <v>704000</v>
+      </c>
+      <c r="Q45" t="str">
         <v>Sudheer Rai</v>
       </c>
-      <c r="O45" t="str">
+      <c r="R45" t="str">
         <v>+91 9800000610</v>
       </c>
-      <c r="P45" t="str">
+      <c r="S45" t="str">
         <v>CBI</v>
       </c>
-      <c r="Q45" t="str">
+      <c r="T45" t="str">
         <v>1075835628</v>
       </c>
-      <c r="R45" t="str">
+      <c r="U45" t="str">
         <v>CBIN0281467</v>
       </c>
-      <c r="S45" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹704000) - Clear</v>
+      <c r="V45" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹704000) - Clear</v>
       </c>
     </row>
     <row r="46">
@@ -3120,23 +3528,32 @@
       <c r="M46">
         <v>608000</v>
       </c>
-      <c r="N46" t="str">
+      <c r="N46">
+        <v>16000</v>
+      </c>
+      <c r="O46">
+        <v>38</v>
+      </c>
+      <c r="P46">
+        <v>608000</v>
+      </c>
+      <c r="Q46" t="str">
         <v>Sita Mathur</v>
       </c>
-      <c r="O46" t="str">
+      <c r="R46" t="str">
         <v>+91 9800000613</v>
       </c>
-      <c r="P46" t="str">
+      <c r="S46" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q46" t="str">
+      <c r="T46" t="str">
         <v>4955000100039329</v>
       </c>
-      <c r="R46" t="str">
+      <c r="U46" t="str">
         <v>PUNB0495500</v>
       </c>
-      <c r="S46" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹608000) - Completed</v>
+      <c r="V46" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹608000) - Completed</v>
       </c>
     </row>
     <row r="47">
@@ -3179,23 +3596,32 @@
       <c r="M47">
         <v>608000</v>
       </c>
-      <c r="N47" t="str">
+      <c r="N47">
+        <v>16000</v>
+      </c>
+      <c r="O47">
+        <v>38</v>
+      </c>
+      <c r="P47">
+        <v>608000</v>
+      </c>
+      <c r="Q47" t="str">
         <v>Sita Mathur</v>
       </c>
-      <c r="O47" t="str">
+      <c r="R47" t="str">
         <v>+91 9800000613</v>
       </c>
-      <c r="P47" t="str">
+      <c r="S47" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q47" t="str">
+      <c r="T47" t="str">
         <v>4955000100039329</v>
       </c>
-      <c r="R47" t="str">
+      <c r="U47" t="str">
         <v>PUNB0495500</v>
       </c>
-      <c r="S47" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹608000) - Completed</v>
+      <c r="V47" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹608000) - Completed</v>
       </c>
     </row>
     <row r="48">
@@ -3238,23 +3664,32 @@
       <c r="M48">
         <v>512000</v>
       </c>
-      <c r="N48" t="str">
+      <c r="N48">
+        <v>16000</v>
+      </c>
+      <c r="O48">
+        <v>32</v>
+      </c>
+      <c r="P48">
+        <v>512000</v>
+      </c>
+      <c r="Q48" t="str">
         <v>Ganga Ram Ganglani</v>
       </c>
-      <c r="O48" t="str">
+      <c r="R48" t="str">
         <v>+91 9800000614</v>
       </c>
-      <c r="P48" t="str">
+      <c r="S48" t="str">
         <v>SBI</v>
       </c>
-      <c r="Q48" t="str">
+      <c r="T48" t="str">
         <v>32261305101</v>
       </c>
-      <c r="R48" t="str">
+      <c r="U48" t="str">
         <v>SBIN0001892</v>
       </c>
-      <c r="S48" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹512000) - neeraj ji</v>
+      <c r="V48" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹512000) - neeraj ji</v>
       </c>
     </row>
     <row r="49">
@@ -3297,22 +3732,31 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="N49" t="str">
+      <c r="N49">
+        <v>0</v>
+      </c>
+      <c r="O49">
+        <v>0</v>
+      </c>
+      <c r="P49">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="str">
         <v>Vimal Tripathi &amp; Namita Tripathi</v>
       </c>
-      <c r="O49" t="str">
+      <c r="R49" t="str">
         <v>+91 9800000701</v>
       </c>
-      <c r="P49" t="str">
+      <c r="S49" t="str">
         <v>SBI</v>
       </c>
-      <c r="Q49" t="str">
+      <c r="T49" t="str">
         <v>51042472748</v>
       </c>
-      <c r="R49" t="str">
+      <c r="U49" t="str">
         <v>SBIN0032479</v>
       </c>
-      <c r="S49" t="str">
+      <c r="V49" t="str">
         <v>Resold title to Vimal Tripathi &amp; Namita Tripathi</v>
       </c>
     </row>
@@ -3356,23 +3800,32 @@
       <c r="M50">
         <v>648000</v>
       </c>
-      <c r="N50" t="str">
+      <c r="N50">
+        <v>16000</v>
+      </c>
+      <c r="O50">
+        <v>40</v>
+      </c>
+      <c r="P50">
+        <v>648000</v>
+      </c>
+      <c r="Q50" t="str">
         <v>Rashmi Rekha Sahu</v>
       </c>
-      <c r="O50" t="str">
+      <c r="R50" t="str">
         <v>+91 9800000703</v>
       </c>
-      <c r="P50" t="str">
+      <c r="S50" t="str">
         <v>UBI</v>
       </c>
-      <c r="Q50" t="str">
+      <c r="T50" t="str">
         <v>520291020167895</v>
       </c>
-      <c r="R50" t="str">
+      <c r="U50" t="str">
         <v>UBIN0929051</v>
       </c>
-      <c r="S50" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹648000) - Clear</v>
+      <c r="V50" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹648000) - Clear</v>
       </c>
     </row>
     <row r="51">
@@ -3415,23 +3868,32 @@
       <c r="M51">
         <v>648000</v>
       </c>
-      <c r="N51" t="str">
+      <c r="N51">
+        <v>16000</v>
+      </c>
+      <c r="O51">
+        <v>40</v>
+      </c>
+      <c r="P51">
+        <v>648000</v>
+      </c>
+      <c r="Q51" t="str">
         <v>Nirmala Devi</v>
       </c>
-      <c r="O51" t="str">
+      <c r="R51" t="str">
         <v>+91 9800000703</v>
       </c>
-      <c r="P51" t="str">
+      <c r="S51" t="str">
         <v>UBI</v>
       </c>
-      <c r="Q51" t="str">
+      <c r="T51" t="str">
         <v>520291020167895</v>
       </c>
-      <c r="R51" t="str">
+      <c r="U51" t="str">
         <v>UBIN0929051</v>
       </c>
-      <c r="S51" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹648000) - Clear</v>
+      <c r="V51" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹648000) - Clear</v>
       </c>
     </row>
     <row r="52">
@@ -3474,23 +3936,32 @@
       <c r="M52">
         <v>704000</v>
       </c>
-      <c r="N52" t="str">
+      <c r="N52">
+        <v>16000</v>
+      </c>
+      <c r="O52">
+        <v>44</v>
+      </c>
+      <c r="P52">
+        <v>704000</v>
+      </c>
+      <c r="Q52" t="str">
         <v>Smita Chauhan</v>
       </c>
-      <c r="O52" t="str">
+      <c r="R52" t="str">
         <v>+91 9800000707</v>
       </c>
-      <c r="P52" t="str">
+      <c r="S52" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q52" t="str">
+      <c r="T52" t="str">
         <v>156701000213</v>
       </c>
-      <c r="R52" t="str">
+      <c r="U52" t="str">
         <v>ICIC0001567</v>
       </c>
-      <c r="S52" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹704000) - Clear</v>
+      <c r="V52" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹704000) - Clear</v>
       </c>
     </row>
     <row r="53">
@@ -3533,23 +4004,32 @@
       <c r="M53">
         <v>1600000</v>
       </c>
-      <c r="N53" t="str">
+      <c r="N53">
+        <v>16000</v>
+      </c>
+      <c r="O53">
+        <v>100</v>
+      </c>
+      <c r="P53">
+        <v>1600000</v>
+      </c>
+      <c r="Q53" t="str">
         <v>Varsha Gupta</v>
       </c>
-      <c r="O53" t="str">
+      <c r="R53" t="str">
         <v>+91 9800000708</v>
       </c>
-      <c r="P53" t="str">
+      <c r="S53" t="str">
         <v>BOI</v>
       </c>
-      <c r="Q53" t="str">
+      <c r="T53" t="str">
         <v>673710310000284</v>
       </c>
-      <c r="R53" t="str">
+      <c r="U53" t="str">
         <v>BKID0006737</v>
       </c>
-      <c r="S53" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V53" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="54">
@@ -3592,23 +4072,32 @@
       <c r="M54">
         <v>1600000</v>
       </c>
-      <c r="N54" t="str">
+      <c r="N54">
+        <v>16000</v>
+      </c>
+      <c r="O54">
+        <v>100</v>
+      </c>
+      <c r="P54">
+        <v>1600000</v>
+      </c>
+      <c r="Q54" t="str">
         <v>Monika Sharma</v>
       </c>
-      <c r="O54" t="str">
+      <c r="R54" t="str">
         <v>+91 9800000708</v>
       </c>
-      <c r="P54" t="str">
+      <c r="S54" t="str">
         <v>BOI</v>
       </c>
-      <c r="Q54" t="str">
+      <c r="T54" t="str">
         <v>673710310000284</v>
       </c>
-      <c r="R54" t="str">
+      <c r="U54" t="str">
         <v>BKID0006737</v>
       </c>
-      <c r="S54" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Clear</v>
+      <c r="V54" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Clear</v>
       </c>
     </row>
     <row r="55">
@@ -3651,23 +4140,32 @@
       <c r="M55">
         <v>544000</v>
       </c>
-      <c r="N55" t="str">
+      <c r="N55">
+        <v>16000</v>
+      </c>
+      <c r="O55">
+        <v>34</v>
+      </c>
+      <c r="P55">
+        <v>544000</v>
+      </c>
+      <c r="Q55" t="str">
         <v>Kushum Shrivastva</v>
       </c>
-      <c r="O55" t="str">
+      <c r="R55" t="str">
         <v>+91 9800000714</v>
       </c>
-      <c r="P55" t="str">
+      <c r="S55" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q55" t="str">
+      <c r="T55" t="str">
         <v>628201528497</v>
       </c>
-      <c r="R55" t="str">
+      <c r="U55" t="str">
         <v>ICIC0006282</v>
       </c>
-      <c r="S55" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹544000) - Completed</v>
+      <c r="V55" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹544000) - Completed</v>
       </c>
     </row>
     <row r="56">
@@ -3710,23 +4208,32 @@
       <c r="M56">
         <v>544000</v>
       </c>
-      <c r="N56" t="str">
+      <c r="N56">
+        <v>16000</v>
+      </c>
+      <c r="O56">
+        <v>34</v>
+      </c>
+      <c r="P56">
+        <v>544000</v>
+      </c>
+      <c r="Q56" t="str">
         <v>Manish Sharma</v>
       </c>
-      <c r="O56" t="str">
+      <c r="R56" t="str">
         <v>+91 9800000714</v>
       </c>
-      <c r="P56" t="str">
+      <c r="S56" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q56" t="str">
+      <c r="T56" t="str">
         <v>628201528497</v>
       </c>
-      <c r="R56" t="str">
+      <c r="U56" t="str">
         <v>ICIC0006282</v>
       </c>
-      <c r="S56" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹544000) - Completed</v>
+      <c r="V56" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹544000) - Completed</v>
       </c>
     </row>
     <row r="57">
@@ -3769,23 +4276,32 @@
       <c r="M57">
         <v>674000</v>
       </c>
-      <c r="N57" t="str">
+      <c r="N57">
+        <v>16000</v>
+      </c>
+      <c r="O57">
+        <v>42.125</v>
+      </c>
+      <c r="P57">
+        <v>674000</v>
+      </c>
+      <c r="Q57" t="str">
         <v>Bhawna Babbar</v>
       </c>
-      <c r="O57" t="str">
+      <c r="R57" t="str">
         <v>+91 9800000801</v>
       </c>
-      <c r="P57" t="str">
+      <c r="S57" t="str">
         <v>HDFC</v>
       </c>
-      <c r="Q57" t="str">
+      <c r="T57" t="str">
         <v>50100046289562</v>
       </c>
-      <c r="R57" t="str">
+      <c r="U57" t="str">
         <v>HDFC0000439</v>
       </c>
-      <c r="S57" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹674000) - Completed</v>
+      <c r="V57" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹674000) - Completed</v>
       </c>
     </row>
     <row r="58">
@@ -3828,23 +4344,32 @@
       <c r="M58">
         <v>674000</v>
       </c>
-      <c r="N58" t="str">
+      <c r="N58">
+        <v>16000</v>
+      </c>
+      <c r="O58">
+        <v>42.125</v>
+      </c>
+      <c r="P58">
+        <v>674000</v>
+      </c>
+      <c r="Q58" t="str">
         <v>Mohini Choudhary</v>
       </c>
-      <c r="O58" t="str">
+      <c r="R58" t="str">
         <v>+91 9800000801</v>
       </c>
-      <c r="P58" t="str">
+      <c r="S58" t="str">
         <v>HDFC</v>
       </c>
-      <c r="Q58" t="str">
+      <c r="T58" t="str">
         <v>50100046289562</v>
       </c>
-      <c r="R58" t="str">
+      <c r="U58" t="str">
         <v>HDFC0000439</v>
       </c>
-      <c r="S58" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹674000) - Completed</v>
+      <c r="V58" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹674000) - Completed</v>
       </c>
     </row>
     <row r="59">
@@ -3887,23 +4412,32 @@
       <c r="M59">
         <v>688000</v>
       </c>
-      <c r="N59" t="str">
+      <c r="N59">
+        <v>16000</v>
+      </c>
+      <c r="O59">
+        <v>43</v>
+      </c>
+      <c r="P59">
+        <v>688000</v>
+      </c>
+      <c r="Q59" t="str">
         <v>Anita Gautam</v>
       </c>
-      <c r="O59" t="str">
+      <c r="R59" t="str">
         <v>+91 9800000813</v>
       </c>
-      <c r="P59" t="str">
+      <c r="S59" t="str">
         <v>CNB</v>
       </c>
-      <c r="Q59" t="str">
+      <c r="T59" t="str">
         <v>2946101050158</v>
       </c>
-      <c r="R59" t="str">
+      <c r="U59" t="str">
         <v>CNRB0002946</v>
       </c>
-      <c r="S59" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹688000) - neeraj ji</v>
+      <c r="V59" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹688000) - neeraj ji</v>
       </c>
     </row>
     <row r="60">
@@ -3946,23 +4480,32 @@
       <c r="M60">
         <v>672000</v>
       </c>
-      <c r="N60" t="str">
+      <c r="N60">
+        <v>16000</v>
+      </c>
+      <c r="O60">
+        <v>42</v>
+      </c>
+      <c r="P60">
+        <v>672000</v>
+      </c>
+      <c r="Q60" t="str">
         <v>Ashok Kumar Agarwal</v>
       </c>
-      <c r="O60" t="str">
+      <c r="R60" t="str">
         <v>+91 9800000814</v>
       </c>
-      <c r="P60" t="str">
+      <c r="S60" t="str">
         <v>UBI</v>
       </c>
-      <c r="Q60" t="str">
+      <c r="T60" t="str">
         <v>540002010000522</v>
       </c>
-      <c r="R60" t="str">
+      <c r="U60" t="str">
         <v>UBIN0554006</v>
       </c>
-      <c r="S60" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹672000) - Completed</v>
+      <c r="V60" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹672000) - Completed</v>
       </c>
     </row>
     <row r="61">
@@ -4005,22 +4548,31 @@
       <c r="M61">
         <v>146788</v>
       </c>
-      <c r="N61" t="str">
+      <c r="N61">
+        <v>20972</v>
+      </c>
+      <c r="O61">
+        <v>6</v>
+      </c>
+      <c r="P61">
+        <v>146788</v>
+      </c>
+      <c r="Q61" t="str">
         <v>Satyajeet Sharma</v>
       </c>
-      <c r="O61" t="str">
+      <c r="R61" t="str">
         <v>+91 9800000906</v>
       </c>
-      <c r="P61" t="str">
+      <c r="S61" t="str">
         <v>BOI</v>
       </c>
-      <c r="Q61" t="str">
+      <c r="T61" t="str">
         <v>685410110001041</v>
       </c>
-      <c r="R61" t="str">
+      <c r="U61" t="str">
         <v>BKID0006854</v>
       </c>
-      <c r="S61" t="str">
+      <c r="V61" t="str">
         <v>Historical title archive</v>
       </c>
     </row>
@@ -4064,23 +4616,32 @@
       <c r="M62">
         <v>624000</v>
       </c>
-      <c r="N62" t="str">
+      <c r="N62">
+        <v>16000</v>
+      </c>
+      <c r="O62">
+        <v>39</v>
+      </c>
+      <c r="P62">
+        <v>624000</v>
+      </c>
+      <c r="Q62" t="str">
         <v>Ravi Shankar Venkatrama</v>
       </c>
-      <c r="O62" t="str">
+      <c r="R62" t="str">
         <v>+91 9800000907</v>
       </c>
-      <c r="P62" t="str">
+      <c r="S62" t="str">
         <v>CBI</v>
       </c>
-      <c r="Q62" t="str">
+      <c r="T62" t="str">
         <v>3463518978</v>
       </c>
-      <c r="R62" t="str">
+      <c r="U62" t="str">
         <v>CBIN0284592</v>
       </c>
-      <c r="S62" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹624000) - Completed</v>
+      <c r="V62" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹624000) - Completed</v>
       </c>
     </row>
     <row r="63">
@@ -4123,23 +4684,32 @@
       <c r="M63">
         <v>624000</v>
       </c>
-      <c r="N63" t="str">
+      <c r="N63">
+        <v>16000</v>
+      </c>
+      <c r="O63">
+        <v>39</v>
+      </c>
+      <c r="P63">
+        <v>624000</v>
+      </c>
+      <c r="Q63" t="str">
         <v>Sikha Srivastav</v>
       </c>
-      <c r="O63" t="str">
+      <c r="R63" t="str">
         <v>+91 9800000907</v>
       </c>
-      <c r="P63" t="str">
+      <c r="S63" t="str">
         <v>CBI</v>
       </c>
-      <c r="Q63" t="str">
+      <c r="T63" t="str">
         <v>3463518978</v>
       </c>
-      <c r="R63" t="str">
+      <c r="U63" t="str">
         <v>CBIN0284592</v>
       </c>
-      <c r="S63" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹624000) - Completed</v>
+      <c r="V63" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹624000) - Completed</v>
       </c>
     </row>
     <row r="64">
@@ -4182,23 +4752,32 @@
       <c r="M64">
         <v>1600000</v>
       </c>
-      <c r="N64" t="str">
+      <c r="N64">
+        <v>16000</v>
+      </c>
+      <c r="O64">
+        <v>100</v>
+      </c>
+      <c r="P64">
+        <v>1600000</v>
+      </c>
+      <c r="Q64" t="str">
         <v>Ekta Sharma</v>
       </c>
-      <c r="O64" t="str">
+      <c r="R64" t="str">
         <v>+91 9800000908</v>
       </c>
-      <c r="P64" t="str">
+      <c r="S64" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q64" t="str">
+      <c r="T64" t="str">
         <v>008301513260</v>
       </c>
-      <c r="R64" t="str">
+      <c r="U64" t="str">
         <v>ICIC0000083</v>
       </c>
-      <c r="S64" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Completed</v>
+      <c r="V64" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Completed</v>
       </c>
     </row>
     <row r="65">
@@ -4241,23 +4820,32 @@
       <c r="M65">
         <v>512000</v>
       </c>
-      <c r="N65" t="str">
+      <c r="N65">
+        <v>16000</v>
+      </c>
+      <c r="O65">
+        <v>32</v>
+      </c>
+      <c r="P65">
+        <v>512000</v>
+      </c>
+      <c r="Q65" t="str">
         <v>Pallavi Gupta</v>
       </c>
-      <c r="O65" t="str">
+      <c r="R65" t="str">
         <v>+91 9800000913</v>
       </c>
-      <c r="P65" t="str">
+      <c r="S65" t="str">
         <v>PNB</v>
       </c>
-      <c r="Q65" t="str">
+      <c r="T65" t="str">
         <v>2961000200118101</v>
       </c>
-      <c r="R65" t="str">
+      <c r="U65" t="str">
         <v>PUNB0296100</v>
       </c>
-      <c r="S65" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹512000) - bank</v>
+      <c r="V65" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹512000) - bank</v>
       </c>
     </row>
     <row r="66">
@@ -4300,23 +4888,32 @@
       <c r="M66">
         <v>1600000</v>
       </c>
-      <c r="N66" t="str">
+      <c r="N66">
+        <v>16000</v>
+      </c>
+      <c r="O66">
+        <v>100</v>
+      </c>
+      <c r="P66">
+        <v>1600000</v>
+      </c>
+      <c r="Q66" t="str">
         <v>Raj Minocha</v>
       </c>
-      <c r="O66" t="str">
+      <c r="R66" t="str">
         <v>+91 9800001003</v>
       </c>
-      <c r="P66" t="str">
+      <c r="S66" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q66" t="str">
+      <c r="T66" t="str">
         <v>083101001596</v>
       </c>
-      <c r="R66" t="str">
+      <c r="U66" t="str">
         <v>ICIC0000831</v>
       </c>
-      <c r="S66" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Completed</v>
+      <c r="V66" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Completed</v>
       </c>
     </row>
     <row r="67">
@@ -4359,23 +4956,32 @@
       <c r="M67">
         <v>1600000</v>
       </c>
-      <c r="N67" t="str">
+      <c r="N67">
+        <v>16000</v>
+      </c>
+      <c r="O67">
+        <v>100</v>
+      </c>
+      <c r="P67">
+        <v>1600000</v>
+      </c>
+      <c r="Q67" t="str">
         <v>Rimpi Rani</v>
       </c>
-      <c r="O67" t="str">
+      <c r="R67" t="str">
         <v>+91 9800001003</v>
       </c>
-      <c r="P67" t="str">
+      <c r="S67" t="str">
         <v>ICICI</v>
       </c>
-      <c r="Q67" t="str">
+      <c r="T67" t="str">
         <v>083101001596</v>
       </c>
-      <c r="R67" t="str">
+      <c r="U67" t="str">
         <v>ICIC0000831</v>
       </c>
-      <c r="S67" t="str">
-        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Paid ₹1600000) - Completed</v>
+      <c r="V67" t="str">
+        <v>100-Mo Pre-Possession Contract (@ ₹16000/mo, Total Rent Paid ₹1600000) - Completed</v>
       </c>
     </row>
     <row r="68">
@@ -4418,28 +5024,37 @@
       <c r="M68">
         <v>0</v>
       </c>
-      <c r="N68" t="str">
+      <c r="N68">
+        <v>0</v>
+      </c>
+      <c r="O68">
+        <v>0</v>
+      </c>
+      <c r="P68">
+        <v>0</v>
+      </c>
+      <c r="Q68" t="str">
         <v>Vijay Rani</v>
       </c>
-      <c r="O68" t="str">
+      <c r="R68" t="str">
         <v>+91 9800001104</v>
       </c>
-      <c r="P68" t="str">
+      <c r="S68" t="str">
         <v/>
       </c>
-      <c r="Q68" t="str">
+      <c r="T68" t="str">
         <v/>
       </c>
-      <c r="R68" t="str">
+      <c r="U68" t="str">
         <v/>
       </c>
-      <c r="S68" t="str">
+      <c r="V68" t="str">
         <v>Resold title to Vijay Rani</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V68"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>